<commit_message>
Add Microsoft customer segment field (Corporate/Enterprise/SMB)
Adds MS Segment as a mandatory dropdown column on the Cards sheet
(values sourced from the Lists sheet) and wires it into the HTML
gallery: card meta line, sidebar filter, detail modal, and search.
</commit_message>
<xml_diff>
--- a/battle-cards.xlsx
+++ b/battle-cards.xlsx
@@ -18,7 +18,7 @@
     <sheet name="Lists" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Cards!$A$3:$AA$500</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Cards!$A$3:$AB$500</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -503,7 +503,7 @@
     <t>Closed lists</t>
   </si>
   <si>
-    <t>Industry, country, ranges, workloads and statuses come from the Lists sheet. Adding a value there is a deliberate act - filtering only stays useful if the lists stay closed.</t>
+    <t>Industry, country, ranges, workloads, segment and statuses come from the Lists sheet. Adding a value there is a deliberate act - filtering only stays useful if the lists stay closed.</t>
   </si>
   <si>
     <t>Reference Status has no default</t>
@@ -1808,7 +1808,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AA28"/>
+  <dimension ref="A1:AB28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1828,6 +1828,7 @@
     <col min="25" max="25" width="12" customWidth="1"/>
     <col min="26" max="26" width="14" customWidth="1"/>
     <col min="27" max="27" width="22" customWidth="1"/>
+    <col min="28" max="28" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -1840,7 +1841,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:27" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:28" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="14" t="s">
         <v>46</v>
       </c>
@@ -1922,8 +1923,13 @@
       <c r="AA3" s="15" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="4" spans="1:27" ht="46" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB3" s="14" t="inlineStr">
+        <is>
+          <t>MS Segment *</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" spans="1:28" ht="46" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="16" t="s">
         <v>73</v>
       </c>
@@ -1999,8 +2005,13 @@
       <c r="AA4" s="16" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="5" spans="1:27" ht="46" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB4" s="16" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" spans="1:28" ht="46" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="16" t="s">
         <v>93</v>
       </c>
@@ -2070,8 +2081,13 @@
       <c r="AA5" s="16" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="6" spans="1:27" ht="46" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB5" s="16" t="inlineStr">
+        <is>
+          <t>Corporate</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="1:28" ht="46" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="16" t="s">
         <v>107</v>
       </c>
@@ -2147,8 +2163,13 @@
       <c r="AA6" s="16" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="7" spans="1:27" ht="46" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB6" s="16" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" spans="1:28" ht="46" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="16" t="s">
         <v>121</v>
       </c>
@@ -2220,8 +2241,13 @@
       <c r="AA7" s="16" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="8" spans="1:27" ht="46" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB7" s="16" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" spans="1:28" ht="46" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="16" t="s">
         <v>132</v>
       </c>
@@ -2291,8 +2317,13 @@
       <c r="AA8" s="16" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="9" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB8" s="16" t="inlineStr">
+        <is>
+          <t>Corporate</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="17"/>
       <c r="B9" s="17"/>
       <c r="C9" s="17"/>
@@ -2320,8 +2351,9 @@
       <c r="Y9" s="17"/>
       <c r="Z9" s="17"/>
       <c r="AA9" s="17"/>
-    </row>
-    <row r="10" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB9" s="17"/>
+    </row>
+    <row r="10" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="17"/>
       <c r="B10" s="17"/>
       <c r="C10" s="17"/>
@@ -2349,8 +2381,9 @@
       <c r="Y10" s="17"/>
       <c r="Z10" s="17"/>
       <c r="AA10" s="17"/>
-    </row>
-    <row r="11" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB10" s="17"/>
+    </row>
+    <row r="11" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="17"/>
       <c r="B11" s="17"/>
       <c r="C11" s="17"/>
@@ -2378,8 +2411,9 @@
       <c r="Y11" s="17"/>
       <c r="Z11" s="17"/>
       <c r="AA11" s="17"/>
-    </row>
-    <row r="12" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB11" s="17"/>
+    </row>
+    <row r="12" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="17"/>
       <c r="B12" s="17"/>
       <c r="C12" s="17"/>
@@ -2407,8 +2441,9 @@
       <c r="Y12" s="17"/>
       <c r="Z12" s="17"/>
       <c r="AA12" s="17"/>
-    </row>
-    <row r="13" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB12" s="17"/>
+    </row>
+    <row r="13" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="17"/>
       <c r="B13" s="17"/>
       <c r="C13" s="17"/>
@@ -2436,8 +2471,9 @@
       <c r="Y13" s="17"/>
       <c r="Z13" s="17"/>
       <c r="AA13" s="17"/>
-    </row>
-    <row r="14" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB13" s="17"/>
+    </row>
+    <row r="14" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="17"/>
       <c r="B14" s="17"/>
       <c r="C14" s="17"/>
@@ -2465,8 +2501,9 @@
       <c r="Y14" s="17"/>
       <c r="Z14" s="17"/>
       <c r="AA14" s="17"/>
-    </row>
-    <row r="15" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB14" s="17"/>
+    </row>
+    <row r="15" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="17"/>
       <c r="B15" s="17"/>
       <c r="C15" s="17"/>
@@ -2494,8 +2531,9 @@
       <c r="Y15" s="17"/>
       <c r="Z15" s="17"/>
       <c r="AA15" s="17"/>
-    </row>
-    <row r="16" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB15" s="17"/>
+    </row>
+    <row r="16" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="17"/>
       <c r="B16" s="17"/>
       <c r="C16" s="17"/>
@@ -2523,8 +2561,9 @@
       <c r="Y16" s="17"/>
       <c r="Z16" s="17"/>
       <c r="AA16" s="17"/>
-    </row>
-    <row r="17" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB16" s="17"/>
+    </row>
+    <row r="17" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="17"/>
       <c r="B17" s="17"/>
       <c r="C17" s="17"/>
@@ -2552,8 +2591,9 @@
       <c r="Y17" s="17"/>
       <c r="Z17" s="17"/>
       <c r="AA17" s="17"/>
-    </row>
-    <row r="18" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB17" s="17"/>
+    </row>
+    <row r="18" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="17"/>
       <c r="B18" s="17"/>
       <c r="C18" s="17"/>
@@ -2581,8 +2621,9 @@
       <c r="Y18" s="17"/>
       <c r="Z18" s="17"/>
       <c r="AA18" s="17"/>
-    </row>
-    <row r="19" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB18" s="17"/>
+    </row>
+    <row r="19" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="17"/>
       <c r="B19" s="17"/>
       <c r="C19" s="17"/>
@@ -2610,8 +2651,9 @@
       <c r="Y19" s="17"/>
       <c r="Z19" s="17"/>
       <c r="AA19" s="17"/>
-    </row>
-    <row r="20" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB19" s="17"/>
+    </row>
+    <row r="20" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="17"/>
       <c r="B20" s="17"/>
       <c r="C20" s="17"/>
@@ -2639,8 +2681,9 @@
       <c r="Y20" s="17"/>
       <c r="Z20" s="17"/>
       <c r="AA20" s="17"/>
-    </row>
-    <row r="21" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB20" s="17"/>
+    </row>
+    <row r="21" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="17"/>
       <c r="B21" s="17"/>
       <c r="C21" s="17"/>
@@ -2668,8 +2711,9 @@
       <c r="Y21" s="17"/>
       <c r="Z21" s="17"/>
       <c r="AA21" s="17"/>
-    </row>
-    <row r="22" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB21" s="17"/>
+    </row>
+    <row r="22" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="17"/>
       <c r="B22" s="17"/>
       <c r="C22" s="17"/>
@@ -2697,8 +2741,9 @@
       <c r="Y22" s="17"/>
       <c r="Z22" s="17"/>
       <c r="AA22" s="17"/>
-    </row>
-    <row r="23" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB22" s="17"/>
+    </row>
+    <row r="23" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="17"/>
       <c r="B23" s="17"/>
       <c r="C23" s="17"/>
@@ -2726,8 +2771,9 @@
       <c r="Y23" s="17"/>
       <c r="Z23" s="17"/>
       <c r="AA23" s="17"/>
-    </row>
-    <row r="24" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB23" s="17"/>
+    </row>
+    <row r="24" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="17"/>
       <c r="B24" s="17"/>
       <c r="C24" s="17"/>
@@ -2755,8 +2801,9 @@
       <c r="Y24" s="17"/>
       <c r="Z24" s="17"/>
       <c r="AA24" s="17"/>
-    </row>
-    <row r="25" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB24" s="17"/>
+    </row>
+    <row r="25" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="17"/>
       <c r="B25" s="17"/>
       <c r="C25" s="17"/>
@@ -2784,8 +2831,9 @@
       <c r="Y25" s="17"/>
       <c r="Z25" s="17"/>
       <c r="AA25" s="17"/>
-    </row>
-    <row r="26" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB25" s="17"/>
+    </row>
+    <row r="26" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="17"/>
       <c r="B26" s="17"/>
       <c r="C26" s="17"/>
@@ -2813,8 +2861,9 @@
       <c r="Y26" s="17"/>
       <c r="Z26" s="17"/>
       <c r="AA26" s="17"/>
-    </row>
-    <row r="27" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB26" s="17"/>
+    </row>
+    <row r="27" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="17"/>
       <c r="B27" s="17"/>
       <c r="C27" s="17"/>
@@ -2842,8 +2891,9 @@
       <c r="Y27" s="17"/>
       <c r="Z27" s="17"/>
       <c r="AA27" s="17"/>
-    </row>
-    <row r="28" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB27" s="17"/>
+    </row>
+    <row r="28" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="17"/>
       <c r="B28" s="17"/>
       <c r="C28" s="17"/>
@@ -2871,9 +2921,10 @@
       <c r="Y28" s="17"/>
       <c r="Z28" s="17"/>
       <c r="AA28" s="17"/>
+      <c r="AB28" s="17"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:AA500" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A3:AB500" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <dataValidations count="3">
     <dataValidation type="textLength" errorStyle="warning" operator="lessThanOrEqual" allowBlank="1" errorTitle="Summary too long" error="The summary is longer than 600 characters. It will still render, but it may overflow the card." sqref="L4:L500" xr:uid="{00000000-0002-0000-0100-00000C000000}">
       <formula1>600</formula1>
@@ -2893,7 +2944,7 @@
   <legacyDrawing r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="12">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="13">
         <x14:dataValidation type="list" allowBlank="1" errorTitle="Value not in the list" error="Pick a value from the dropdown. To add a new one, put it on the Lists sheet first." promptTitle="HQ Country" prompt="Pick from the list." xr:uid="{00000000-0002-0000-0100-000000000000}">
           <x14:formula1>
             <xm:f>Lists!$B$5:$B$51</xm:f>
@@ -2966,6 +3017,12 @@
           </x14:formula1>
           <xm:sqref>Y4:Y500</xm:sqref>
         </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" errorTitle="Value not in the list" error="Pick a value from the dropdown. To add a new one, put it on the Lists sheet first." promptTitle="MS Segment" prompt="Pick from the list. Corporate, Enterprise or SMB." xr:uid="{00000000-0002-0000-0100-00000F000000}">
+          <x14:formula1>
+            <xm:f>Lists!$I$5:$I$7</xm:f>
+          </x14:formula1>
+          <xm:sqref>AB4:AB500</xm:sqref>
+        </x14:dataValidation>
       </x14:dataValidations>
     </ext>
   </extLst>
@@ -2974,7 +3031,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
@@ -2984,6 +3041,7 @@
     <col min="6" max="6" width="19" customWidth="1"/>
     <col min="7" max="7" width="13" customWidth="1"/>
     <col min="8" max="8" width="11" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
@@ -2996,7 +3054,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="22" t="s">
         <v>144</v>
       </c>
@@ -3021,8 +3079,13 @@
       <c r="H4" s="22" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I4" s="22" t="inlineStr">
+        <is>
+          <t>MS Segment</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="23" t="s">
         <v>96</v>
       </c>
@@ -3047,8 +3110,13 @@
       <c r="H5" s="23" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I5" s="23" t="inlineStr">
+        <is>
+          <t>SMB</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="23" t="s">
         <v>124</v>
       </c>
@@ -3073,8 +3141,13 @@
       <c r="H6" s="23" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I6" s="23" t="inlineStr">
+        <is>
+          <t>Corporate</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="23" t="s">
         <v>76</v>
       </c>
@@ -3089,6 +3162,11 @@
       </c>
       <c r="E7" s="23" t="s">
         <v>157</v>
+      </c>
+      <c r="I7" s="23" t="inlineStr">
+        <is>
+          <t>Enterprise</t>
+        </is>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Add Short Description column to battle cards
Adds a free-text Short Description field to the Cards sheet and
renders it centered on each card between the divider and the stats
row, so a one- or two-sentence case summary shows without opening
the detail view.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/battle-cards.xlsx
+++ b/battle-cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucassantacruz/Library/CloudStorage/GoogleDrive-lpsantacruz@gmail.com/My Drive/lpsanbr Repository/Battle_Card/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1AD0C95-CEAA-A649-8DE9-6DDC5A7393DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FCE6924-446B-9645-A7BF-F25B9D1427D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19920" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -381,7 +381,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="212">
   <si>
     <t>BATTLE CARDS   |   one row = one card</t>
   </si>
@@ -1011,6 +1011,12 @@
   </si>
   <si>
     <t>https://www.enat.receita.economia.gov.br/pt-br/area_nacional/noticias/logo-rfb/image_preview</t>
+  </si>
+  <si>
+    <t>Short Description</t>
+  </si>
+  <si>
+    <t>Descreva aqui!</t>
   </si>
 </sst>
 </file>
@@ -2819,7 +2825,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:O993"/>
+  <dimension ref="A1:P993"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="28.5" customWidth="1"/>
@@ -2831,19 +2837,20 @@
     <col min="12" max="12" width="18" customWidth="1"/>
     <col min="13" max="14" width="34" customWidth="1"/>
     <col min="15" max="15" width="22" customWidth="1"/>
+    <col min="16" max="16" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
@@ -2889,8 +2896,11 @@
       <c r="O3" s="5" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P3" s="5" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="11" t="s">
         <v>147</v>
       </c>
@@ -2930,8 +2940,11 @@
       <c r="O4" s="11" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P4" s="11" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
         <v>149</v>
       </c>
@@ -2971,8 +2984,11 @@
       <c r="O5" s="11" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P5" s="11" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
         <v>51</v>
       </c>
@@ -3014,8 +3030,11 @@
       <c r="O6" s="11" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P6" s="11" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="23" t="s">
         <v>180</v>
       </c>
@@ -3059,8 +3078,11 @@
       <c r="O7" s="25" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P7" s="11" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="22" t="s">
         <v>152</v>
       </c>
@@ -3100,8 +3122,11 @@
       <c r="O8" s="11" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P8" s="11" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="23" t="s">
         <v>172</v>
       </c>
@@ -3141,8 +3166,11 @@
       <c r="O9" s="23" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P9" s="11" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
         <v>161</v>
       </c>
@@ -3182,8 +3210,11 @@
       <c r="O10" s="11" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="11" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P10" s="11" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="11" t="s">
         <v>207</v>
       </c>
@@ -3225,8 +3256,11 @@
       <c r="O11" s="11" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="12" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P11" s="11" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="23" t="s">
         <v>185</v>
       </c>
@@ -3270,8 +3304,11 @@
       <c r="O12" s="23" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="13" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P12" s="11" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="11" t="s">
         <v>171</v>
       </c>
@@ -3311,8 +3348,11 @@
       <c r="O13" s="11" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="14" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P13" s="11" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="23" t="s">
         <v>188</v>
       </c>
@@ -3352,8 +3392,11 @@
       <c r="O14" s="25" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="15" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P14" s="11" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="23" t="s">
         <v>176</v>
       </c>
@@ -3397,8 +3440,11 @@
       <c r="O15" s="25" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="16" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P15" s="11" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="11" t="s">
         <v>113</v>
       </c>
@@ -3438,8 +3484,11 @@
       <c r="O16" s="11" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="17" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P16" s="11" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="35" t="s">
         <v>195</v>
       </c>
@@ -3477,8 +3526,11 @@
       <c r="O17" s="11" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="18" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P17" s="11" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="25" t="s">
         <v>192</v>
       </c>
@@ -3518,8 +3570,11 @@
       <c r="O18" s="25" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="19" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P18" s="11" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="26" t="s">
         <v>158</v>
       </c>
@@ -3559,8 +3614,11 @@
       <c r="O19" s="27" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="20" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P19" s="11" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="26" t="s">
         <v>155</v>
       </c>
@@ -3600,8 +3658,11 @@
       <c r="O20" s="27" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="21" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P20" s="11" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="24" t="s">
         <v>162</v>
       </c>
@@ -3641,8 +3702,11 @@
       <c r="O21" s="27" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="22" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P21" s="11" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="24" t="s">
         <v>168</v>
       </c>
@@ -3684,8 +3748,11 @@
       <c r="O22" s="27" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="23" spans="1:15" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P22" s="11" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="24" t="s">
         <v>164</v>
       </c>
@@ -3729,8 +3796,11 @@
       <c r="O23" s="27" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="24" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P23" s="11" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
       <c r="E24" s="3"/>
@@ -3742,7 +3812,7 @@
       <c r="L24" s="3"/>
       <c r="O24" s="3"/>
     </row>
-    <row r="25" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
@@ -3754,7 +3824,7 @@
       <c r="L25" s="3"/>
       <c r="O25" s="3"/>
     </row>
-    <row r="26" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
       <c r="E26" s="3"/>
@@ -3766,7 +3836,7 @@
       <c r="L26" s="3"/>
       <c r="O26" s="3"/>
     </row>
-    <row r="27" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
@@ -3778,7 +3848,7 @@
       <c r="L27" s="3"/>
       <c r="O27" s="3"/>
     </row>
-    <row r="28" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
@@ -3790,7 +3860,7 @@
       <c r="L28" s="3"/>
       <c r="O28" s="3"/>
     </row>
-    <row r="29" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
@@ -3802,7 +3872,7 @@
       <c r="L29" s="3"/>
       <c r="O29" s="3"/>
     </row>
-    <row r="30" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
       <c r="E30" s="3"/>
@@ -3814,7 +3884,7 @@
       <c r="L30" s="3"/>
       <c r="O30" s="3"/>
     </row>
-    <row r="31" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
@@ -3826,7 +3896,7 @@
       <c r="L31" s="3"/>
       <c r="O31" s="3"/>
     </row>
-    <row r="32" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>

</xml_diff>